<commit_message>
add update remover duplicatas len >= 150 novas consultas
</commit_message>
<xml_diff>
--- a/erros.xlsx
+++ b/erros.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t xml:space="preserve">cnpj</t>
   </si>
@@ -44,48 +44,6 @@
   </si>
   <si>
     <t xml:space="preserve">cnae_desc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05.957.149/0001-87</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05.958.128/0001-86</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05.958.357/0001-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05.958.971/0001-62</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05.959.479/0001-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05.959.604/0001-83</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05.959.931/0001-35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05.960.053/0001-78</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05.960.071/0001-50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05.960.415/0001-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05.960.589/0001-93</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05.960.876/0001-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05.960.902/0001-93</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05.961.048/0001-80</t>
   </si>
 </sst>
 </file>
@@ -412,87 +370,45 @@
       <c r="K1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>8</v>
-      </c>
       <c r="F2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>9</v>
-      </c>
       <c r="F3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>10</v>
-      </c>
       <c r="F4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>11</v>
-      </c>
       <c r="F5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>12</v>
-      </c>
       <c r="F6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>13</v>
-      </c>
       <c r="F7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>14</v>
-      </c>
       <c r="F8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="F9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>16</v>
-      </c>
       <c r="F10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>17</v>
-      </c>
       <c r="F11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>18</v>
-      </c>
       <c r="F12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>19</v>
-      </c>
       <c r="F13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>20</v>
-      </c>
       <c r="F14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>21</v>
-      </c>
       <c r="F15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
add novos dados na base
</commit_message>
<xml_diff>
--- a/erros.xlsx
+++ b/erros.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
   <si>
     <t>cnpj</t>
   </si>
@@ -49,16 +49,43 @@
     <t>06.009.235/0001-20</t>
   </si>
   <si>
+    <t>06.020.049/0001-92</t>
+  </si>
+  <si>
+    <t>06.029.385/0001-04</t>
+  </si>
+  <si>
+    <t>06.879.489/0001-08</t>
+  </si>
+  <si>
     <t>2025-07-15 12:28:34</t>
   </si>
   <si>
     <t>2025-07-15 12:29:27</t>
   </si>
   <si>
+    <t>2025-07-15 14:37:00</t>
+  </si>
+  <si>
+    <t>2025-07-15 14:37:15</t>
+  </si>
+  <si>
+    <t>2025-07-18 13:29:57</t>
+  </si>
+  <si>
     <t>('Connection aborted.', RemoteDisconnected('Remote end closed connection without response'))</t>
   </si>
   <si>
     <t>Falha após 3 tentativas ou erro desconhecido</t>
+  </si>
+  <si>
+    <t>HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06020049000192 (Caused by NewConnectionError('&lt;urllib3.connection.HTTPSConnection object at 0x71f77f914e80&gt;: Failed to establish a new connection: [Errno -3] Temporary failure in name resolution'))</t>
+  </si>
+  <si>
+    <t>HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Read timed out. (read timeout=29)</t>
+  </si>
+  <si>
+    <t>HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Read timed out. (read timeout=35)</t>
   </si>
 </sst>
 </file>
@@ -416,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -456,10 +483,10 @@
         <v>10</v>
       </c>
       <c r="I2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J2" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -467,10 +494,54 @@
         <v>10</v>
       </c>
       <c r="I3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="J3" t="s">
-        <v>14</v>
+      <c r="I5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="I6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I7" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
atualizados script erros e add checkpoint erros
</commit_message>
<xml_diff>
--- a/erros.xlsx
+++ b/erros.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="98">
   <si>
     <t xml:space="preserve">cnpj</t>
   </si>
@@ -50,6 +50,270 @@
   </si>
   <si>
     <t xml:space="preserve">erro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">05.940.084/0001-67</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-07-30 10:41:59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/05940084000167 (Caused by NameResolutionError("&lt;urllib3.connection.HTTPSConnection object at 0x77e7cf217b10&gt;: Failed to resolve 'publica.cnpj.ws' ([Errno -3] Temporary failure in name resolution)"))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.047.718/0001-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-07-30 17:06:12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Falha após 3 tentativas ou erro desconhecido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.061.275/0001-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-07-30 17:57:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Read timed out. (read timeout=35)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.087.635/0001-54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-07-31 08:54:58</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06087635000154 (Caused by NameResolutionError("&lt;urllib3.connection.HTTPSConnection object at 0x778df091ec10&gt;: Failed to resolve 'publica.cnpj.ws' ([Errno -3] Temporary failure in name resolution)"))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.088.000/0001-71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-07-31 08:57:31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">502 Server Error: Bad Gateway for url: https://publica.cnpj.ws/cnpj/06088000000171</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-07-31 08:57:42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.095.466/0001-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-07-31 09:27:41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06095466000102 (Caused by NameResolutionError("&lt;urllib3.connection.HTTPSConnection object at 0x778df091ec10&gt;: Failed to resolve 'publica.cnpj.ws' ([Errno -3] Temporary failure in name resolution)"))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.100.103/0001-00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-07-31 09:43:14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06100103000100 (Caused by NameResolutionError("&lt;urllib3.connection.HTTPSConnection object at 0x778df091fc50&gt;: Failed to resolve 'publica.cnpj.ws' ([Errno -3] Temporary failure in name resolution)"))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.104.282/0001-53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-07-31 10:02:19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06104282000153 (Caused by NameResolutionError("&lt;urllib3.connection.HTTPSConnection object at 0x778df05ed310&gt;: Failed to resolve 'publica.cnpj.ws' ([Errno -3] Temporary failure in name resolution)"))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.107.009/0001-82</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-07-31 10:17:45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06107009000182 (Caused by NameResolutionError("&lt;urllib3.connection.HTTPSConnection object at 0x7cf2309aefd0&gt;: Failed to resolve 'publica.cnpj.ws' ([Errno -3] Temporary failure in name resolution)"))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.235.668/0001-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-07-31 18:19:16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">522 Server Error:  for url: https://publica.cnpj.ws/cnpj/06235668000102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.262.185/0001-99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 09:06:19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06262185000199 (Caused by NameResolutionError("&lt;urllib3.connection.HTTPSConnection object at 0x77a1f16aead0&gt;: Failed to resolve 'publica.cnpj.ws' ([Errno -3] Temporary failure in name resolution)"))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.265.671/0001-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 09:17:04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06265671000160 (Caused by NameResolutionError("&lt;urllib3.connection.HTTPSConnection object at 0x77a1f16ae5d0&gt;: Failed to resolve 'publica.cnpj.ws' ([Errno -3] Temporary failure in name resolution)"))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 09:17:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.272.613/0001-64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 09:41:11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06272613000164 (Caused by NameResolutionError("&lt;urllib3.connection.HTTPSConnection object at 0x77a1f16af110&gt;: Failed to resolve 'publica.cnpj.ws' ([Errno -3] Temporary failure in name resolution)"))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.307.350/0001-81</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 11:35:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">('Connection aborted.', RemoteDisconnected('Remote end closed connection without response'))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.311.795/0001-35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 11:51:53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06311795000135 (Caused by ConnectTimeoutError(&lt;urllib3.connection.HTTPSConnection object at 0x7b0fe2762e90&gt;, 'Connection to publica.cnpj.ws timed out. (connect timeout=35)'))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 11:53:16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06311795000135 (Caused by ConnectTimeoutError(&lt;urllib3.connection.HTTPSConnection object at 0x7b0fe2762710&gt;, 'Connection to publica.cnpj.ws timed out. (connect timeout=35)'))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 11:53:29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.322.201/0001-91</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 12:25:42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">('Connection aborted.', ConnectionResetError(104, 'Connection reset by peer'))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.322.738/0001-51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 12:29:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.323.592/0001-69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 12:32:34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.324.942/0001-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 12:36:44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.325.886/0001-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 12:37:53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.326.025/0001-66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 12:40:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06326025000166 (Caused by ConnectTimeoutError(&lt;urllib3.connection.HTTPSConnection object at 0x7b0fe2761bd0&gt;, 'Connection to publica.cnpj.ws timed out. (connect timeout=35)'))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.338.924/0001-89</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 13:22:08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.371.607/0001-64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 14:38:14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06371607000164 (Caused by ConnectTimeoutError(&lt;urllib3.connection.HTTPSConnection object at 0x7b0fe2761450&gt;, 'Connection to publica.cnpj.ws timed out. (connect timeout=35)'))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 14:39:37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06371607000164 (Caused by ConnectTimeoutError(&lt;urllib3.connection.HTTPSConnection object at 0x7b0fe2761bd0&gt;, 'Connection to publica.cnpj.ws timed out. (connect timeout=35)'))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 14:39:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.496.111/0001-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 15:00:42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.538.588/0001-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 15:13:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06538588000118 (Caused by ConnectTimeoutError(&lt;urllib3.connection.HTTPSConnection object at 0x7b0fe2761310&gt;, 'Connection to publica.cnpj.ws timed out. (connect timeout=35)'))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.539.248/0001-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 15:15:04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 15:17:02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPSConnectionPool(host='publica.cnpj.ws', port=443): Max retries exceeded with url: /cnpj/06539248000101 (Caused by ConnectTimeoutError(&lt;urllib3.connection.HTTPSConnection object at 0x7b0fe2761450&gt;, 'Connection to publica.cnpj.ws timed out. (connect timeout=35)'))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 15:17:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.555.274/0001-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 15:27:36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06.604.714/0001-95</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 15:37:08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01 16:02:41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">400 Client Error: Bad Request for url: https://publica.cnpj.ws/cnpj/00000000000</t>
   </si>
 </sst>
 </file>
@@ -85,9 +349,8 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="Cambria"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -341,7 +604,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -376,9 +639,423 @@
         <v>9</v>
       </c>
     </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="0" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" s="0" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="0" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="0" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="J6" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="J7" s="0" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="I8" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="0" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="J9" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="J10" s="0" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="I11" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="J11" s="0" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="I12" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="J12" s="0" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="I13" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="J13" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="I14" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="J14" s="0" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="I15" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="J15" s="0" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="I16" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="J16" s="0" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="I17" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="J17" s="0" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="I18" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="J18" s="0" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="I19" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="J19" s="0" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="I20" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="J20" s="0" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="I21" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="J21" s="0" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="I22" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="J22" s="0" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="I23" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="J23" s="0" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="I24" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="J24" s="0" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="I25" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="J25" s="0" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="I26" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="J26" s="0" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="I27" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="J27" s="0" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="I28" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="J28" s="0" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="I29" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="J29" s="0" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="I30" s="0" t="s">
+        <v>81</v>
+      </c>
+      <c r="J30" s="0" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="I31" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="J31" s="0" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="I32" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="J32" s="0" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="I33" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="J33" s="0" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="I34" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="J34" s="0" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="I35" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="J35" s="0" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="I36" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="J36" s="0" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="I37" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="J37" s="0" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="I38" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="J38" s="0" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>

</xml_diff>